<commit_message>
Refresh downloadable manager Excel with confirmed tenure dates
</commit_message>
<xml_diff>
--- a/assets/manager-introductions.xlsx
+++ b/assets/manager-introductions.xlsx
@@ -600,11 +600,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="yyyy/m/d"/>
   </numFmts>
   <fonts count="27">
     <font>
@@ -1465,7 +1466,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -1540,6 +1541,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -2103,14 +2113,22 @@
       <c r="A2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>6</v>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6年金融从业经验，其中5年投资经验。上海财经大学经济学学士、国际商务硕士、北卡罗莱纳大学夏洛特分校数理金融硕士、FRM。
+现任国泰海通资管多资产策略投资部（公募）基金经理，历任国泰海通资管固定收益部研究员、投资经理助理，固定收益投资部基金经理；东证期货衍生品研究院高级金融工程分析师。
+拥有丰富的量化投资策略开发经验，擅长运用主观和定量结合的投资体系，采用自上而下的投研框架进行全局配置管理。</t>
+        </is>
       </c>
       <c r="C2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="12"/>
+      <c r="D2" s="25">
+        <v>44095</v>
+      </c>
+      <c r="E2" s="26">
+        <v>44477</v>
+      </c>
     </row>
     <row r="3" ht="74" customHeight="1" spans="1:5">
       <c r="A3" s="13" t="s">
@@ -2129,8 +2147,12 @@
       <c r="A4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>12</v>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11年证券从业经验，其中7年权益投资经验，东南大学国际经济与贸易学士，南京大学产业经济学硕士。
+现任国泰海通资管综合策略投资部基金经理，历任海通资管权益投资二部投资经理助理、权益二部投资经理、公募权益部总监助理。
+具有多年行业研究和权益投资工作经验，投资追求价值与成长的平衡，尊重产业发展的周期规律，挖掘符合时代特征的投资机会，顺势而为，长线投资。</t>
+        </is>
       </c>
       <c r="C4" s="10"/>
       <c r="D4" s="16">
@@ -2150,8 +2172,12 @@
       <c r="C5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
+      <c r="D5" s="27">
+        <v>41152</v>
+      </c>
+      <c r="E5" s="27">
+        <v>42384</v>
+      </c>
     </row>
     <row r="6" ht="68" customHeight="1" spans="1:5">
       <c r="A6" s="13" t="s">
@@ -2163,8 +2189,12 @@
       <c r="C6" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
+      <c r="D6" s="27">
+        <v>42633</v>
+      </c>
+      <c r="E6" s="27">
+        <v>43843</v>
+      </c>
     </row>
     <row r="7" ht="86" customHeight="1" spans="1:5">
       <c r="A7" s="13" t="s">
@@ -2176,8 +2206,12 @@
       <c r="C7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
+      <c r="D7" s="27">
+        <v>41534</v>
+      </c>
+      <c r="E7" s="27">
+        <v>41534</v>
+      </c>
     </row>
     <row r="8" ht="74" customHeight="1" spans="1:5">
       <c r="A8" s="13" t="s">
@@ -2194,12 +2228,20 @@
       <c r="A9" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="17" t="s">
-        <v>25</v>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12年证券研究投资经验，其中9年固定收益投资经验。复旦大学金融硕士。
+现任国泰海通资管固定收益投资部（公募）副总经理，固定收益投资部（公募）基金经理。
+组合管理注重细致谋划、灵活应对，曾管理过多种类型和风格的固收产品，擅长流动性分析和捕捉宏观周期驱动的趋势性机会，注重收益的同时兼具出色的风险控制能力。</t>
+        </is>
       </c>
       <c r="C9" s="10"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
+      <c r="D9" s="27">
+        <v>41868</v>
+      </c>
+      <c r="E9" s="27">
+        <v>42935</v>
+      </c>
     </row>
     <row r="10" ht="72" customHeight="1" spans="1:5">
       <c r="A10" s="18" t="s">
@@ -2220,23 +2262,39 @@
       <c r="A11" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="17" t="s">
-        <v>29</v>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2年中国债券市场投资经验。上海交通大学经济学学士、复旦大学硕士研究生。
+现任国泰海通资管固定收益投资部（公募）副总经理、基金经理。
+长期从事机构自营投资及追求绝对收益型资管产品的投资管理，擅长宏观利率交易以及多资产视角下的绝对收益投资。</t>
+        </is>
       </c>
       <c r="C11" s="10"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
+      <c r="D11" s="27">
+        <v>42240</v>
+      </c>
+      <c r="E11" s="27">
+        <v>45237</v>
+      </c>
     </row>
     <row r="12" ht="93" customHeight="1" spans="1:5">
       <c r="A12" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="17" t="s">
-        <v>31</v>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6年证券从业经验，其中5年投资经验。法国巴黎第九大学计量经济学博士，特许金融分析师。
+现任国泰海通资管综合策略投资部投资经理，从事全球大类资产相关投资研究工作。加入国泰海通资管之前，曾就职于法国Credit Agricole SA（东方汇理银行总行）、前海联合基金、某国内头部券商自营交易台（一级场外衍生品交易商），历任金融工程师、量化研究员、投资经理等职
+拥有严谨的数据分析建模框架，成熟的量化投资体系；投研交易经验覆盖：欧美货币基金赎回行为建模、利率衍生品交易、国债期货量化策略、可转债套利策略、股票深度学习端到端模型、商品CTA策略、全球大类资产配置策略。</t>
+        </is>
       </c>
       <c r="C12" s="10"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
+      <c r="D12" s="27">
+        <v>44091</v>
+      </c>
+      <c r="E12" s="27">
+        <v>44280</v>
+      </c>
     </row>
     <row r="13" ht="60" customHeight="1" spans="1:5">
       <c r="A13" s="18" t="s">
@@ -2246,19 +2304,31 @@
         <v>33</v>
       </c>
       <c r="C13" s="10"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
+      <c r="D13" s="27">
+        <v>44553</v>
+      </c>
+      <c r="E13" s="27">
+        <v>43342</v>
+      </c>
     </row>
     <row r="14" ht="81" customHeight="1" spans="1:5">
       <c r="A14" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>35</v>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9年证券从业经验，其中1年投资经验。厦门大学金融工程专业博士，上海交通大学金融工程方向博士后。
+现任国泰海通资管综合策略投资部投资经理，主要从事场外衍生品和结构性产品的研究创新与投资工作。历任申万宏源证券、国投证券产品设计总监、销售交易与风险管理工作。
+深耕衍生品全价值链，擅长运用量化模型构建创新产品框架，主导设计并落地多款结构性产品，在复杂衍生品定价、投资组合管理及结构化产品创新领域具有深厚积累。</t>
+        </is>
       </c>
       <c r="C14" s="10"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
+      <c r="D14" s="27">
+        <v>42995</v>
+      </c>
+      <c r="E14" s="27">
+        <v>45777</v>
+      </c>
     </row>
     <row r="15" ht="60" customHeight="1" spans="1:5">
       <c r="A15" s="13" t="s">
@@ -2270,19 +2340,31 @@
       <c r="C15" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
+      <c r="D15" s="27">
+        <v>43997</v>
+      </c>
+      <c r="E15" s="27">
+        <v>45988</v>
+      </c>
     </row>
     <row r="16" ht="60" customHeight="1" spans="1:5">
       <c r="A16" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="14" t="s">
-        <v>40</v>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18年证券从业经验，其中13年投资经验。中国科学院数学与系统科学研究院概率论与数理统计博士。
+现任国泰海通资管量化投资部（私募）投资经理；历任国泰君安证券衍生产品部研究员、国泰君安证券资产管理总部研究员等职；
+在量化模型等方面有深入研究及丰富投资经验，尤其擅长期权定价与结构化产品设计、对冲、套利及alpha策略、大类资产配置策略等。</t>
+        </is>
       </c>
       <c r="C16" s="10"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
+      <c r="D16" s="27">
+        <v>39468</v>
+      </c>
+      <c r="E16" s="27">
+        <v>41309</v>
+      </c>
     </row>
     <row r="17" ht="60" customHeight="1" spans="1:5">
       <c r="A17" s="13" t="s">
@@ -2344,27 +2426,42 @@
       <c r="A21" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="17" t="s">
-        <v>51</v>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12年证券从业经验，其中6年投资经验。美国杜兰大学金融学硕士。
+现任国泰海通资管固定收益投资部（私募）投资经理，曾任职于光大保德信基金，历任固定收益部研究员与投资经理助理。专注信用增强策略，聚焦君享年华定开系列。</t>
+        </is>
       </c>
       <c r="C21" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
+      <c r="D21" s="27">
+        <v>41881</v>
+      </c>
+      <c r="E21" s="27">
+        <v>44064</v>
+      </c>
     </row>
     <row r="22" ht="93" customHeight="1" spans="1:5">
       <c r="A22" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="17" t="s">
-        <v>54</v>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上海财经大学管理学硕士，9年证券从业经验，1年投资经验。
+现任国泰海通资管固定收益投资部（私募）投资经理；曾就职于新世纪评级、浙商证券资管。历任国泰海通资管信用研究员，投资经理助理，从事信用债研究投资。
+对城投、周期等行业信用评级、信用策略研究和信用债投资具有丰富经验。</t>
+        </is>
       </c>
       <c r="C22" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
+      <c r="D22" s="27">
+        <v>42994</v>
+      </c>
+      <c r="E22" s="27">
+        <v>45726</v>
+      </c>
     </row>
     <row r="23" ht="158" customHeight="1" spans="1:5">
       <c r="A23" s="13" t="s">
@@ -2405,36 +2502,58 @@
       <c r="A26" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="14" t="s">
-        <v>64</v>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8年证券和资管行业从业经验，其中2年投资管理经验。中央财经大学统计学学士、应用统计学硕士。
+现任国泰海通资管综合策略投资部投资经理。历任国泰君安证券数字金融部、私人客户部、申万宏源证券产品与资产配置中心，从事量化策略研究、投研系统建设和组合管理等工作，拥有丰富的宏观研究、策略研究和基金组合管理经验。</t>
+        </is>
       </c>
       <c r="C26" s="10"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
+      <c r="D26" s="27">
+        <v>43353</v>
+      </c>
+      <c r="E26" s="27">
+        <v>45429</v>
+      </c>
     </row>
     <row r="27" ht="90" customHeight="1" spans="1:5">
       <c r="A27" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="17" t="s">
-        <v>65</v>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9年证券从业经验，其中1年投资经验。上海财经大学管理学硕士。
+现任国泰海通资管固定收益投资部（私募）投资经理 。曾就职于新世纪评级、浙商证券资管。历任国泰海通资管信用研究员，投资经理助理，从事信用债研究投资。
+对城投、周期等行业信用评级、信用策略研究和信用债投资具有丰富经验。</t>
+        </is>
       </c>
       <c r="C27" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
+      <c r="D27" s="27">
+        <v>42994</v>
+      </c>
+      <c r="E27" s="27">
+        <v>45726</v>
+      </c>
     </row>
     <row r="28" ht="80" customHeight="1" spans="1:5">
       <c r="A28" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="17" t="s">
-        <v>67</v>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4年信用债投研经验，其中1年投资经验。CPA，英国格拉斯哥大学投资学硕士。
+现任国泰海通资管固定收益投资部投资经理，擅长自下而上信用挖掘和定价，投研经验丰富。先后在中证鹏元、平安资管和国信资管担任信用研究员和投资助理。</t>
+        </is>
       </c>
       <c r="C28" s="10"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
+      <c r="D28" s="27">
+        <v>44833</v>
+      </c>
+      <c r="E28" s="27">
+        <v>45762</v>
+      </c>
     </row>
     <row r="29" ht="73" customHeight="1" spans="1:5">
       <c r="A29" s="18" t="s">
@@ -2453,8 +2572,12 @@
       <c r="A30" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="B30" s="14" t="s">
-        <v>70</v>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14年证券行业固定收益从业经验，其中10年投资经验。上海财经大学金融学硕士。
+现任国泰海通资管固定收益投资部（私募）投资经理；历任海通资管投资经理。
+具备完善的固收领域研究框架和丰富扎实的债券型产品投资管理经验。</t>
+        </is>
       </c>
       <c r="C30" s="10"/>
       <c r="D30" s="16">
@@ -2483,8 +2606,12 @@
       <c r="A32" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B32" s="14" t="s">
-        <v>74</v>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10年证券从业经验，其中6年投资经验。美国伍斯特理工金融数学硕士，武汉大学数理金融试验班学士(金融和数学双学位)。 
+现任国泰海通资管固定收益投资部（私募）投资经理，历任海通资管量化投资部研究员，海通资管专户固定收益部投资经理助理、投资经理。
+对宏观经济、大类资产表现有深入的研究积累，具备较强的风险识别和价值挖掘能力，擅长多资产配置。</t>
+        </is>
       </c>
       <c r="C32" s="10"/>
       <c r="D32" s="16">
@@ -2504,32 +2631,51 @@
       <c r="C33" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D33" s="15"/>
-      <c r="E33" s="15"/>
+      <c r="D33" s="27">
+        <v>42705</v>
+      </c>
+      <c r="E33" s="27">
+        <v>43747</v>
+      </c>
     </row>
     <row r="34" ht="94" customHeight="1" spans="1:5">
       <c r="A34" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="14" t="s">
-        <v>78</v>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6年证券从业经验，其中0年投资经验。美国凯斯西储大学金融风险管理硕士学位，山东大学金融学学士，具备扎实的数理金融与统计分析功底。
+现任国泰海通资管衍生品及结构性产品投资经理。过往任职期间曾主导了多种创新型衍生品、结构性产品及策略的设计与开发，对衍生品定价、衍生品交易策略搭建、衍生品及结构性产品设计具有丰富经验。</t>
+        </is>
       </c>
       <c r="C34" s="10"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
+      <c r="D34" s="27">
+        <v>43997</v>
+      </c>
+      <c r="E34" s="27">
+        <v>45988</v>
+      </c>
     </row>
     <row r="35" ht="80" customHeight="1" spans="1:5">
       <c r="A35" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="B35" s="14" t="s">
-        <v>80</v>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10年债券从业经验，其中6年投资经验。上海交通大学工学学士、金融学硕士。
+现任国泰海通资管固定收益投资部（私募）投资经理。历任国泰君安证券资产管理公司固定收益部信用、转债、大类资产配置研究员以及投资经理助理。
+为行业内较早进行可转债投研的人员，擅长自下而上的基本面分析，深挖个券，兼顾择时，投资风格偏稳健型与价值型。</t>
+        </is>
       </c>
       <c r="C35" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
+      <c r="D35" s="27">
+        <v>42576</v>
+      </c>
+      <c r="E35" s="27">
+        <v>44099</v>
+      </c>
     </row>
     <row r="36" ht="64" customHeight="1" spans="1:5">
       <c r="A36" s="18" t="s">
@@ -2539,15 +2685,23 @@
         <v>83</v>
       </c>
       <c r="C36" s="10"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="15"/>
+      <c r="D36" s="27">
+        <v>44425</v>
+      </c>
+      <c r="E36" s="27">
+        <v>44278</v>
+      </c>
     </row>
     <row r="37" ht="83" customHeight="1" spans="1:5">
       <c r="A37" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B37" s="14" t="s">
-        <v>85</v>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13年从业经验，其中2年证券从业经验，10年投资经验。中央财经大学国民经济学硕士。
+现任固定收益投资部（公募）基金经理，曾就职于平安资产管理有限责任公司、百年保险资产管理有限责任公司。
+具备丰富的宏观分析和大类资产配置经验，重视均衡配置和收益来源的多元化，力求以最小的波动，追求投资性价比最大化。</t>
+        </is>
       </c>
       <c r="C37" s="10" t="s">
         <v>86</v>
@@ -2580,8 +2734,12 @@
       <c r="A39" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="B39" s="14" t="s">
-        <v>91</v>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11年证券从业经验，其中10年固收投资经验。西安交通大学金融学和曼彻斯特大学统计学硕士。
+现任国泰海通资管固定收益投资部（公募）基金经理，历任海通资管固定收益研究员、投资经理助理、投资经理，公募固收部总监、专户固收部总监。
+擅长宏观利率研判和大类资产分析，在波动市场保持相对平稳的运作；具备完善的固收领域研究框架和丰富扎实的债券型产品投资管理经验。</t>
+        </is>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="16">
@@ -2608,8 +2766,12 @@
       <c r="A41" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="14" t="s">
-        <v>96</v>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9年从业经验，其中7年投资经验。北京大学管理学硕士。
+现任国泰海通资管固定收益投资部（公募）基金经理。历任花旗集团新加坡投资银行部分析师，上海海通证券资产管理有限公司固定收益研究部研究员、固定收益三部投资经理、公募固收部基金经理。
+擅长结合自上而下的宏观分析与自下而上的中微观、机构行为分析。具备丰富的账户管理经验。</t>
+        </is>
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="16">
@@ -2623,25 +2785,41 @@
       <c r="A42" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="B42" s="14" t="s">
-        <v>98</v>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3年固收投资及管理经验。中国人民大学经济学硕士；
+历任中国农业银行总行金融市场部债券投资经理、国寿安保基金公司专户投资经理、中金资管投资经理，现任国泰海通证券资产管理有限公司固定收益投资部（北京）基金经理（执行董事）；
+擅长中高评级信用债及可转债投资，具有丰富的组合管理经验及大型资金配置能力。</t>
+        </is>
       </c>
       <c r="C42" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
+      <c r="D42" s="27">
+        <v>44742</v>
+      </c>
+      <c r="E42" s="27">
+        <v>45103</v>
+      </c>
     </row>
     <row r="43" ht="77" customHeight="1" spans="1:5">
       <c r="A43" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="B43" s="14" t="s">
-        <v>101</v>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3年海外及国内固收领域从业经验，3年投资组合管理经验。美国密歇根大学商学院硕士研究生学历，注册金融分析师（CFA)；
+现任国泰海通资管固定收益投资部（北京）总经理。历任法兴银行下属FIMAT集团（纽约）固定收益衍生产品部分析员、法国巴黎银行（纽约）固定收益利率产品部副总裁、董事，法国巴黎银行（香港）执行董事，中再资产管理股份有限公司固定收益部副总经理、资深投资经理I级等职；
+投资风格稳健，对于保险资金大类资产配置及固定收益投资有丰富经验</t>
+        </is>
       </c>
       <c r="C43" s="10"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
+      <c r="D43" s="27">
+        <v>45020</v>
+      </c>
+      <c r="E43" s="27">
+        <v>45163</v>
+      </c>
     </row>
     <row r="44" ht="60" customHeight="1" spans="1:5">
       <c r="A44" s="18" t="s">

</xml_diff>